<commit_message>
fix(ce): page layout, drop internal sheet from the client file
- الـ Matrix بقى في صفحة A3 landscape واحدة، والباقي fit-to-width.
  ده اتعرف لما الملف اترسم لـ PDF واتشاف.
- شيت تعديلات الرسم V2 اتشال من ملف العميل لأنه داخلي، ومكانه ISSUES.md.
- build_ce.py بقى بيكتب في مسار نسبي.
</commit_message>
<xml_diff>
--- a/deliverables/PH-LCP-01-CE_RevA.xlsx
+++ b/deliverables/PH-LCP-01-CE_RevA.xlsx
@@ -11,7 +11,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C&amp;E Matrix" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IO List" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Drawing V2 changes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'C&amp;E Matrix'!$4:$6</definedName>
@@ -553,7 +552,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -578,7 +577,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Purpose</t>
@@ -590,7 +589,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="34" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Scope</t>
@@ -602,7 +601,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="47" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Not in scope (Rev. A)</t>
@@ -615,7 +614,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="56" customHeight="1">
+    <row r="7" ht="47" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Burner flame safety</t>
@@ -627,7 +626,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
+    <row r="8" ht="34" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Hardwired safety</t>
@@ -639,7 +638,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1">
+    <row r="9" ht="34" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Fail-safe outputs</t>
@@ -651,7 +650,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="112" customHeight="1">
+    <row r="10" ht="99" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>How to read the matrix</t>
@@ -666,7 +665,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="34" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Requested from client</t>
@@ -736,6 +735,7 @@
     <mergeCell ref="B6:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2706,7 +2706,7 @@
     <mergeCell ref="F4:F6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2714,7 +2714,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -2937,6 +2937,7 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2944,7 +2945,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4161,175 +4162,6 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>CHANGES FOR DRAWING PH-LCP-01 V2 (internal)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Project: Burner PetroBaker  |  Panel: LCP-01  |  Ref. drawing: PH-LCP-01 V1  |  Document: PH-LCP-01-CE  |  Rev. A (for client review)  |  26-10-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Sheet</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Change</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Reason</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Show PSH-101, LSH-102, LSHH-103 as contacts that OPEN on alarm (de-energise to trip).</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Fail-safe: broken wire = trip. Confirmed by Eng. Ahmed Zain.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Mark I12.5 'scrubber LSL — not installed'.</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Not installed on site.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Sheet title 'DI SM12211' → 'DI SM1221'.</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Typo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>1 / 14</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Page index lists 17 rows; Panel GA refers to 'device list /17' which does not exist. Add sheet 17 or remove the reference.</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Consistency.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>XQ:15–18 are labelled SPARE but R8/R9 drive BR02 stage lamps H5/H6.</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Consistency.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ce): client response columns, filter, sheet protection
- عمودين أصفر للعميل: Client response (قايمة منسدلة Approved /
  Approved with comment / Rejected)، وClient comment.
- باقي الشيت محمي من غير باسورد عشان محدّش يعدّل صف بالغلط،
  والفلتر شغّال (مثلًا Source = PH proposal).
- نسخة PDF في deliverables/ جنب الإكسيل.
</commit_message>
<xml_diff>
--- a/deliverables/PH-LCP-01-CE_RevA.xlsx
+++ b/deliverables/PH-LCP-01-CE_RevA.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IO List" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'C&amp;E Matrix'!$A$6:$S$38</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'C&amp;E Matrix'!$4:$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -60,7 +61,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -104,6 +105,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFFF99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
@@ -139,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -180,10 +186,18 @@
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -665,7 +679,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="34" customHeight="1">
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Requested from client</t>
@@ -673,7 +687,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Review the rows marked 'PH proposal' and confirm or mark up. Parameter values are on sheet 'Parameters' and are adjustable from the HMI.</t>
+          <t>On sheet 'C&amp;E Matrix', fill the two yellow columns for every row: 'Client response' (Approved / Approved with comment / Rejected) and 'Client comment'. Rows marked 'PH proposal' need particular attention. All other cells are protected against accidental edits (no password). Use the filter on the header row, e.g. Source = PH proposal. Parameter values are on sheet 'Parameters' and are adjustable from the HMI.</t>
         </is>
       </c>
     </row>
@@ -745,7 +759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q38"/>
+  <dimension ref="A1:S38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -765,6 +779,8 @@
     <col width="20" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="50" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="40" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -832,6 +848,16 @@
           <t>Remarks</t>
         </is>
       </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>Client response</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>Client comment</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="G5" s="6" t="inlineStr">
@@ -1018,6 +1044,8 @@
           <t>Burners: also cut by hardwired S0 NC2/NC3 (client e-mail: ESD impact on burner ON/OFF). Scrubber valves to safe position on ESD = PH proposal.</t>
         </is>
       </c>
+      <c r="R8" s="14" t="n"/>
+      <c r="S8" s="15" t="n"/>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
@@ -1101,6 +1129,8 @@
           <t>Result of valve types (NO / NO / NC) and relay outputs — no program needed.</t>
         </is>
       </c>
+      <c r="R9" s="14" t="n"/>
+      <c r="S9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -1169,7 +1199,7 @@
           <t>Manual (S2) after cleared</t>
         </is>
       </c>
-      <c r="P11" s="14" t="inlineStr">
+      <c r="P11" s="16" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -1179,6 +1209,8 @@
           <t>Client e-mail: scrubber alarms/trips. Burners NOT tripped (confirmed by Eng. Ahmed Zain).</t>
         </is>
       </c>
+      <c r="R11" s="14" t="n"/>
+      <c r="S11" s="15" t="n"/>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
@@ -1228,7 +1260,7 @@
           <t>Automatic when cleared</t>
         </is>
       </c>
-      <c r="P12" s="14" t="inlineStr">
+      <c r="P12" s="16" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -1238,6 +1270,8 @@
           <t>Pre-alarm before LSHH-103.</t>
         </is>
       </c>
+      <c r="R12" s="14" t="n"/>
+      <c r="S12" s="15" t="n"/>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
@@ -1299,7 +1333,7 @@
           <t>Manual (S2) after cleared</t>
         </is>
       </c>
-      <c r="P13" s="14" t="inlineStr">
+      <c r="P13" s="16" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -1309,6 +1343,8 @@
           <t>Burners NOT tripped (confirmed by Eng. Ahmed Zain).</t>
         </is>
       </c>
+      <c r="R13" s="14" t="n"/>
+      <c r="S13" s="15" t="n"/>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
@@ -1354,7 +1390,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P14" s="14" t="inlineStr">
+      <c r="P14" s="16" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -1364,6 +1400,8 @@
           <t>Not installed — excluded from Rev. A. Input reserved for future use.</t>
         </is>
       </c>
+      <c r="R14" s="14" t="n"/>
+      <c r="S14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -1424,7 +1462,7 @@
           <t>Auto (AUTO mode)</t>
         </is>
       </c>
-      <c r="P16" s="14" t="inlineStr">
+      <c r="P16" s="16" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -1434,6 +1472,8 @@
           <t>Client sheet: burner may start only when level has reached LSL. Contact closes with liquid present, so a broken wire also blocks the burner.</t>
         </is>
       </c>
+      <c r="R16" s="14" t="n"/>
+      <c r="S16" s="15" t="n"/>
     </row>
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
@@ -1487,7 +1527,7 @@
           <t>Auto when T &lt;= SP − HYST (AUTO mode)</t>
         </is>
       </c>
-      <c r="P17" s="14" t="inlineStr">
+      <c r="P17" s="16" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -1497,6 +1537,8 @@
           <t>Client cases 2/3/6. Higher of inlet/outlet is used (PH proposal). Restart after hysteresis avoids short-cycling: each start costs ~50 s of purge.</t>
         </is>
       </c>
+      <c r="R17" s="14" t="n"/>
+      <c r="S17" s="15" t="n"/>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
@@ -1530,7 +1572,7 @@
         </is>
       </c>
       <c r="G18" s="9" t="n"/>
-      <c r="H18" s="15" t="inlineStr">
+      <c r="H18" s="17" t="inlineStr">
         <is>
           <t>RUN</t>
         </is>
@@ -1556,6 +1598,8 @@
           <t>Requests 2nd stage / high fire for fast heat-up. Between 60 and 70 °C: 1st stage only.</t>
         </is>
       </c>
+      <c r="R18" s="14" t="n"/>
+      <c r="S18" s="15" t="n"/>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
@@ -1623,6 +1667,8 @@
           <t>Without a valid temperature the burner cannot be controlled.</t>
         </is>
       </c>
+      <c r="R19" s="14" t="n"/>
+      <c r="S19" s="15" t="n"/>
     </row>
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
@@ -1690,6 +1736,8 @@
           <t>Burner's own control box has already shut the gas valves. PLC removes the heat request so the burner does not restart by itself after a local reset.</t>
         </is>
       </c>
+      <c r="R20" s="14" t="n"/>
+      <c r="S20" s="15" t="n"/>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
@@ -1757,6 +1805,8 @@
           <t>Normal start cycle is ~55 s (RS100 manual §6.8.1) / ~65 s (DLX 53 manual).</t>
         </is>
       </c>
+      <c r="R21" s="14" t="n"/>
+      <c r="S21" s="15" t="n"/>
     </row>
     <row r="22" ht="48" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
@@ -1802,7 +1852,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P22" s="14" t="inlineStr">
+      <c r="P22" s="16" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -1812,6 +1862,8 @@
           <t>Client e-mail: Auto/Manual selection. MAN: operator starts with START and stops with STOP. All trips and the temperature setpoint (C07b) still apply; no automatic restart.</t>
         </is>
       </c>
+      <c r="R22" s="14" t="n"/>
+      <c r="S22" s="15" t="n"/>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
@@ -1844,7 +1896,7 @@
           <t>Command</t>
         </is>
       </c>
-      <c r="G23" s="15" t="inlineStr">
+      <c r="G23" s="17" t="inlineStr">
         <is>
           <t>RUN</t>
         </is>
@@ -1871,6 +1923,8 @@
           <t>MAN: starts the burner. AUTO: re-enables automatic control after STOP. Ignored while any trip or permissive is active.</t>
         </is>
       </c>
+      <c r="R23" s="14" t="n"/>
+      <c r="S23" s="15" t="n"/>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
@@ -1934,6 +1988,8 @@
           <t>Works in AUTO and MAN. In AUTO the burner stays off until START is pressed.</t>
         </is>
       </c>
+      <c r="R24" s="14" t="n"/>
+      <c r="S24" s="15" t="n"/>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
@@ -1997,6 +2053,8 @@
           <t>RS100 is approved for intermittent operation and must stop at least once every 24 h (RS100 manual §5.10).</t>
         </is>
       </c>
+      <c r="R25" s="14" t="n"/>
+      <c r="S25" s="15" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -2057,7 +2115,7 @@
           <t>Auto (AUTO mode)</t>
         </is>
       </c>
-      <c r="P27" s="14" t="inlineStr">
+      <c r="P27" s="16" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -2067,6 +2125,8 @@
           <t>Client sheet: burner may start only when level has reached LSL. Contact closes with liquid present, so a broken wire also blocks the burner.</t>
         </is>
       </c>
+      <c r="R27" s="14" t="n"/>
+      <c r="S27" s="15" t="n"/>
     </row>
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
@@ -2120,7 +2180,7 @@
           <t>Auto when T &lt;= SP − HYST (AUTO mode)</t>
         </is>
       </c>
-      <c r="P28" s="14" t="inlineStr">
+      <c r="P28" s="16" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -2130,6 +2190,8 @@
           <t>Client cases 2/3/6. Higher of inlet/outlet is used (PH proposal). Restart after hysteresis avoids short-cycling: each start costs ~50 s of purge.</t>
         </is>
       </c>
+      <c r="R28" s="14" t="n"/>
+      <c r="S28" s="15" t="n"/>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
@@ -2165,7 +2227,7 @@
       <c r="G29" s="9" t="n"/>
       <c r="H29" s="9" t="n"/>
       <c r="I29" s="9" t="n"/>
-      <c r="J29" s="15" t="inlineStr">
+      <c r="J29" s="17" t="inlineStr">
         <is>
           <t>RUN</t>
         </is>
@@ -2189,6 +2251,8 @@
           <t>Requests 2nd stage / high fire for fast heat-up. Between 60 and 70 °C: 1st stage only.</t>
         </is>
       </c>
+      <c r="R29" s="14" t="n"/>
+      <c r="S29" s="15" t="n"/>
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
@@ -2256,6 +2320,8 @@
           <t>Without a valid temperature the burner cannot be controlled.</t>
         </is>
       </c>
+      <c r="R30" s="14" t="n"/>
+      <c r="S30" s="15" t="n"/>
     </row>
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
@@ -2323,6 +2389,8 @@
           <t>Burner's own control box has already shut the gas valves. PLC removes the heat request so the burner does not restart by itself after a local reset.</t>
         </is>
       </c>
+      <c r="R31" s="14" t="n"/>
+      <c r="S31" s="15" t="n"/>
     </row>
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
@@ -2390,6 +2458,8 @@
           <t>Normal start cycle is ~55 s (RS100 manual §6.8.1) / ~65 s (DLX 53 manual).</t>
         </is>
       </c>
+      <c r="R32" s="14" t="n"/>
+      <c r="S32" s="15" t="n"/>
     </row>
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
@@ -2435,7 +2505,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P33" s="14" t="inlineStr">
+      <c r="P33" s="16" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -2445,6 +2515,8 @@
           <t>Client e-mail: Auto/Manual selection. MAN: operator starts with START and stops with STOP. All trips and the temperature setpoint (C08b) still apply; no automatic restart.</t>
         </is>
       </c>
+      <c r="R33" s="14" t="n"/>
+      <c r="S33" s="15" t="n"/>
     </row>
     <row r="34" ht="36" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
@@ -2479,7 +2551,7 @@
       </c>
       <c r="G34" s="9" t="n"/>
       <c r="H34" s="9" t="n"/>
-      <c r="I34" s="15" t="inlineStr">
+      <c r="I34" s="17" t="inlineStr">
         <is>
           <t>RUN</t>
         </is>
@@ -2504,6 +2576,8 @@
           <t>MAN: starts the burner. AUTO: re-enables automatic control after STOP. Ignored while any trip or permissive is active.</t>
         </is>
       </c>
+      <c r="R34" s="14" t="n"/>
+      <c r="S34" s="15" t="n"/>
     </row>
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
@@ -2567,6 +2641,8 @@
           <t>Works in AUTO and MAN. In AUTO the burner stays off until START is pressed.</t>
         </is>
       </c>
+      <c r="R35" s="14" t="n"/>
+      <c r="S35" s="15" t="n"/>
     </row>
     <row r="36" ht="28" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
@@ -2612,7 +2688,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P36" s="14" t="inlineStr">
+      <c r="P36" s="16" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -2622,6 +2698,8 @@
           <t>Read only: fuel is selected on the burner itself. Shown on HMI.</t>
         </is>
       </c>
+      <c r="R36" s="14" t="n"/>
+      <c r="S36" s="15" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
@@ -2684,27 +2762,38 @@
           <t>Resets latched trips only when their cause has cleared.</t>
         </is>
       </c>
+      <c r="R38" s="14" t="n"/>
+      <c r="S38" s="15" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <autoFilter ref="A6:S38"/>
+  <mergeCells count="19">
     <mergeCell ref="D4:D6"/>
+    <mergeCell ref="A10:S10"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="S4:S6"/>
+    <mergeCell ref="A15:S15"/>
+    <mergeCell ref="F4:F6"/>
+    <mergeCell ref="P4:P6"/>
+    <mergeCell ref="R4:R6"/>
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="A7:S7"/>
     <mergeCell ref="G4:N4"/>
-    <mergeCell ref="A4:A6"/>
     <mergeCell ref="O4:O6"/>
-    <mergeCell ref="P4:P6"/>
-    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="A37:S37"/>
     <mergeCell ref="Q4:Q6"/>
-    <mergeCell ref="A7:Q7"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="A26:Q26"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A37:Q37"/>
-    <mergeCell ref="A15:Q15"/>
-    <mergeCell ref="A10:Q10"/>
-    <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="F4:F6"/>
+    <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A2:S2"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="R8 R9 R11 R12 R13 R14 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose Approved, Approved with comment or Rejected" prompt="Approved / Approved with comment / Rejected" type="list">
+      <formula1>"Approved,Approved with comment,Rejected"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
@@ -2784,7 +2873,7 @@
           <t>Tank temperature setpoint — burner stops at T &gt;= SP</t>
         </is>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="18" t="n">
         <v>70</v>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -2814,7 +2903,7 @@
           <t>Restart hysteresis — burner restarts at T &lt;= SP − HYST</t>
         </is>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="18" t="n">
         <v>5</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -2844,7 +2933,7 @@
           <t>2nd stage / high fire while T &lt; SP − STG</t>
         </is>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="18" t="n">
         <v>10</v>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -2874,7 +2963,7 @@
           <t>Max. time from heat request to RUN feedback</t>
         </is>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8" s="18" t="n">
         <v>120</v>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -2904,7 +2993,7 @@
           <t>Forced stop of BR01 after continuous run</t>
         </is>
       </c>
-      <c r="C9" s="16" t="n">
+      <c r="C9" s="18" t="n">
         <v>24</v>
       </c>
       <c r="D9" s="9" t="inlineStr">

</xml_diff>

<commit_message>
docs: split C&E from the control narrative; close F9–F15
- الـ C&E بقى تريبات وإنذارات وشروط بس (23 صف). الأوضاع والزراير
  والديزل والـ RESET طلعوا منه.
- اتضاف C07g/C08g: البيرنر وقف لوحده وهو شغال.
- E8 بقى HMI alarm بس، لأن H3/H4 متسلّكين على البيرنر مش الـ PLC.
- docs/التشغيل.md: وصف التشغيل بالعربي. الحالات، وAUTO/MAN، وSTART/STOP،
  والـ RESET، ورجوع الكهربا، واللمبات، والشاشة، و10 سيناريوهات اختبار.
- القرارات F10 وF14 وF15 اتاخدت بالأأمن، وزين يقدر يغيّرها.
- F16 جديد: DLX 53 مرحلة واحدة ولا اتنين.
</commit_message>
<xml_diff>
--- a/deliverables/PH-LCP-01-CE_RevA.xlsx
+++ b/deliverables/PH-LCP-01-CE_RevA.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IO List" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'C&amp;E Matrix'!$A$6:$S$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'C&amp;E Matrix'!$A$6:$S$31</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'C&amp;E Matrix'!$4:$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -603,7 +603,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1">
+    <row r="5" ht="47" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Scope</t>
@@ -611,7 +611,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Gas scrubber alarms/trips, ESD, burner BR01 (Riello RS100) and BR02 (DLX 53 SHFP) Auto/Manual control, tank temperature control (client sheet 'Temperature control of burner'), diesel-mode indication.</t>
+          <t>Gas scrubber alarms/trips, ESD, burner BR01 (Riello RS100) and BR02 (DLX 53 SHFP) trips and permissives, tank temperature control (client sheet 'Temperature control of burner'). This matrix lists causes and effects only. Operating modes (AUTO / MAN), START / STOP, RESET, start-up after power loss and lamps are described in the Control Narrative (docs/التشغيل.md).</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
         <is>
           <t>One row per cause. Cells under each effect say what happens to that output while the cause is active. Empty = no action.
 STOP = output de-energised / burner request removed.  RUN = energised.
-OPEN / CLOSE = resulting valve position.  ALARM = HMI alarm and fault lamp.
+OPEN / CLOSE = resulting valve position.  ALARM = HMI alarm (the burner fault lamps H3 / H4 are wired to the burner lockout, not to the PLC).
 Column 'Source' shows where each line comes from: Client = client document; PH proposal = proposed by PH, to be approved by the client.</t>
         </is>
       </c>
@@ -759,7 +759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S38"/>
+  <dimension ref="A1:S31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -905,7 +905,7 @@
       <c r="N5" s="6" t="inlineStr">
         <is>
           <t>E8
-HMI alarm / fault lamp</t>
+HMI alarm</t>
         </is>
       </c>
     </row>
@@ -947,7 +947,7 @@
       </c>
       <c r="N6" s="7" t="inlineStr">
         <is>
-          <t>HMI, H3 / H4</t>
+          <t>HMI</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>Release S0, then S2</t>
+          <t>Release S0, then S2; burners need START</t>
         </is>
       </c>
       <c r="P8" s="13" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="Q8" s="4" t="inlineStr">
         <is>
-          <t>Burners: also cut by hardwired S0 NC2/NC3 (client e-mail: ESD impact on burner ON/OFF). Scrubber valves to safe position on ESD = PH proposal.</t>
+          <t>Burners are also cut by hardwired S0 NC2/NC3 (client e-mail: ESD impact on burner ON/OFF). Scrubber valves to safe position on ESD = PH proposal.</t>
         </is>
       </c>
       <c r="R8" s="14" t="n"/>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>PLC STOP / 24 VDC loss</t>
+          <t>PLC STOP, 24 VDC loss or power-up</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
@@ -1116,7 +1116,7 @@
       <c r="N9" s="9" t="n"/>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>Automatic on restore + S2</t>
+          <t>S2 for scrubber; burners need START</t>
         </is>
       </c>
       <c r="P9" s="13" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="Q9" s="4" t="inlineStr">
         <is>
-          <t>Result of valve types (NO / NO / NC) and relay outputs — no program needed.</t>
+          <t>Result of valve types (NO / NO / NC) and relay outputs. After power returns nothing restarts by itself.</t>
         </is>
       </c>
       <c r="R9" s="14" t="n"/>
@@ -1139,7 +1139,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="48" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
           <t>C03</t>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>Manual (S2) after cleared</t>
+          <t>S2 after cleared</t>
         </is>
       </c>
       <c r="P11" s="16" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="Q11" s="4" t="inlineStr">
         <is>
-          <t>Client e-mail: scrubber alarms/trips. Burners NOT tripped (confirmed by Eng. Ahmed Zain).</t>
+          <t>Client e-mail: scrubber alarms/trips. Burners are NOT tripped (decision PH / Eng. Ahmed Zain); if gas pressure to the burner drops, the burner's own gas pressure switch stops it (C07g / C08g).</t>
         </is>
       </c>
       <c r="R11" s="14" t="n"/>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>Manual (S2) after cleared</t>
+          <t>S2 after cleared</t>
         </is>
       </c>
       <c r="P13" s="16" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="Q13" s="4" t="inlineStr">
         <is>
-          <t>Burners NOT tripped (confirmed by Eng. Ahmed Zain).</t>
+          <t>Burners are NOT tripped (as C03).</t>
         </is>
       </c>
       <c r="R13" s="14" t="n"/>
@@ -1406,7 +1406,7 @@
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>BURNER BR01 — tank TK01</t>
+          <t>BURNER BR01 — tank TK01   (operating modes, START / STOP: see Control Narrative)</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1423,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>TK01 level below low level switch (not ready)</t>
+          <t>TK01 level below low level switch</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
@@ -1459,7 +1459,7 @@
       <c r="N16" s="9" t="n"/>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>Auto (AUTO mode)</t>
+          <t>Automatic when level returns</t>
         </is>
       </c>
       <c r="P16" s="16" t="inlineStr">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="Q16" s="4" t="inlineStr">
         <is>
-          <t>Client sheet: burner may start only when level has reached LSL. Contact closes with liquid present, so a broken wire also blocks the burner.</t>
+          <t>Client sheet: burner may run only when level has reached LSL. Contact closes with liquid present, so a broken wire also blocks the burner.</t>
         </is>
       </c>
       <c r="R16" s="14" t="n"/>
@@ -1498,7 +1498,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>T &gt;= SP (70 °C)</t>
+          <t>max(T) &gt;= SP (70 °C)</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -1524,7 +1524,7 @@
       <c r="N17" s="9" t="n"/>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>Auto when T &lt;= SP − HYST (AUTO mode)</t>
+          <t>Automatic at max(T) &lt;= SP − HYST (65 °C)</t>
         </is>
       </c>
       <c r="P17" s="16" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="Q17" s="4" t="inlineStr">
         <is>
-          <t>Client cases 2/3/6. Higher of inlet/outlet is used (PH proposal). Restart after hysteresis avoids short-cycling: each start costs ~50 s of purge.</t>
+          <t>Client cases 2/3/6. The higher of inlet/outlet is used and the 5 °C restart band are PH proposals: each restart costs ~50 s of purge.</t>
         </is>
       </c>
       <c r="R17" s="14" t="n"/>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>TK01 oil temperature below 2nd-stage threshold</t>
+          <t>TK01 oil temperature low — fast heat-up</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>T &lt; SP − STG (60 °C)</t>
+          <t>max(T) &lt; SP − STG (60 °C)</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
@@ -1585,7 +1585,7 @@
       <c r="N18" s="9" t="n"/>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>Auto when T &gt;= SP − STG</t>
+          <t>Automatic at max(T) &gt;= 60 °C</t>
         </is>
       </c>
       <c r="P18" s="13" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="Q18" s="4" t="inlineStr">
         <is>
-          <t>Requests 2nd stage / high fire for fast heat-up. Between 60 and 70 °C: 1st stage only.</t>
+          <t>2nd stage / high fire. Between 60 and 70 °C the burner runs on 1st stage.</t>
         </is>
       </c>
       <c r="R18" s="14" t="n"/>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Thermocouple fault (wire break / out of range)</t>
+          <t>Thermocouple fault — either of the two</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>SM 1231 diagnostic or value out of range</t>
+          <t>Wire break or value out of range</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>Manual (S2) after fault cleared</t>
+          <t>S2 after fault cleared</t>
         </is>
       </c>
       <c r="P19" s="13" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="Q19" s="4" t="inlineStr">
         <is>
-          <t>Without a valid temperature the burner cannot be controlled.</t>
+          <t>Either sensor failing stops the burner: without both readings the higher value cannot be trusted.</t>
         </is>
       </c>
       <c r="R19" s="14" t="n"/>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>BR01 burner lockout (flame failure, ignition failure, air pressure)</t>
+          <t>BR01 lockout (flame / ignition / air pressure failure)</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
@@ -1693,12 +1693,12 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Lockout relay energised</t>
+          <t>Lockout signal present</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Alarm</t>
+          <t>Trip</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="Q20" s="4" t="inlineStr">
         <is>
-          <t>Burner's own control box has already shut the gas valves. PLC removes the heat request so the burner does not restart by itself after a local reset.</t>
+          <t>The burner's own control box has already closed the gas valves. PLC removes the heat request so the burner does not restart by itself after a local reset.</t>
         </is>
       </c>
       <c r="R20" s="14" t="n"/>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Heat request ON and no RUN feedback within T_START (120 s)</t>
+          <t>Heat request ON, no RUN within T_START (120 s)</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>Manual (S2)</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="P21" s="13" t="inlineStr">
@@ -1802,13 +1802,13 @@
       </c>
       <c r="Q21" s="4" t="inlineStr">
         <is>
-          <t>Normal start cycle is ~55 s (RS100 manual §6.8.1) / ~65 s (DLX 53 manual).</t>
+          <t>RUN = gas valves energised (firing). Normal start ~55 s (RS100 §6.8.1) / ~65 s (DLX 53).</t>
         </is>
       </c>
       <c r="R21" s="14" t="n"/>
       <c r="S21" s="15" t="n"/>
     </row>
-    <row r="22" ht="48" customHeight="1">
+    <row r="22" ht="36" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
           <t>C07g</t>
@@ -1816,56 +1816,68 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>BR01 selector in MANUAL</t>
+          <t>BR01 stopped by itself while running</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>I12.1</t>
+          <t>I0.3</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Selector open = MAN</t>
+          <t>RUN lost, no lockout, heat request still ON</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Mode</t>
-        </is>
-      </c>
-      <c r="G22" s="9" t="n"/>
-      <c r="H22" s="9" t="n"/>
+          <t>Trip</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
       <c r="I22" s="9" t="n"/>
       <c r="J22" s="9" t="n"/>
       <c r="K22" s="9" t="n"/>
       <c r="L22" s="9" t="n"/>
       <c r="M22" s="9" t="n"/>
-      <c r="N22" s="9" t="n"/>
+      <c r="N22" s="12" t="inlineStr">
+        <is>
+          <t>ALARM</t>
+        </is>
+      </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P22" s="16" t="inlineStr">
-        <is>
-          <t>Client</t>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="P22" s="13" t="inlineStr">
+        <is>
+          <t>PH proposal</t>
         </is>
       </c>
       <c r="Q22" s="4" t="inlineStr">
         <is>
-          <t>Client e-mail: Auto/Manual selection. MAN: operator starts with START and stops with STOP. All trips and the temperature setpoint (C07b) still apply; no automatic restart.</t>
+          <t>E.g. safety thermostat TS, gas pressure switch, burner supply lost. Without this row the PLC would keep requesting heat from a burner that is no longer firing.</t>
         </is>
       </c>
       <c r="R22" s="14" t="n"/>
       <c r="S22" s="15" t="n"/>
     </row>
-    <row r="23" ht="36" customHeight="1">
+    <row r="23" ht="28" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
           <t>C07h</t>
@@ -1873,35 +1885,39 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>BR01 START push button (MAN mode)</t>
+          <t>BR01 running continuously for 24 h</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>I0.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Pressed</t>
+          <t>Run timer &gt;= 24 h</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>Command</t>
-        </is>
-      </c>
-      <c r="G23" s="17" t="inlineStr">
-        <is>
-          <t>RUN</t>
-        </is>
-      </c>
-      <c r="H23" s="9" t="n"/>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
       <c r="I23" s="9" t="n"/>
       <c r="J23" s="9" t="n"/>
       <c r="K23" s="9" t="n"/>
@@ -1910,7 +1926,7 @@
       <c r="N23" s="9" t="n"/>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Automatic (restarts on next demand)</t>
         </is>
       </c>
       <c r="P23" s="13" t="inlineStr">
@@ -1920,190 +1936,186 @@
       </c>
       <c r="Q23" s="4" t="inlineStr">
         <is>
-          <t>MAN: starts the burner. AUTO: re-enables automatic control after STOP. Ignored while any trip or permissive is active.</t>
+          <t>RS100 is approved for intermittent operation and must stop at least once every 24 h (RS100 manual §5.10).</t>
         </is>
       </c>
       <c r="R23" s="14" t="n"/>
       <c r="S23" s="15" t="n"/>
     </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>C07i</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>S3</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>BR01 STOP push button</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>I0.6</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Pressed</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>Command</t>
-        </is>
-      </c>
-      <c r="G24" s="10" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>BURNER BR02 — tank TK02   (operating modes, START / STOP: see Control Narrative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>C08a</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>LSL-TK02</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>TK02 level below low level switch</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>I1.3</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>LSL not reached (contact open)</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>Permissive</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="n"/>
+      <c r="H25" s="9" t="n"/>
+      <c r="I25" s="10" t="inlineStr">
         <is>
           <t>STOP</t>
         </is>
       </c>
-      <c r="H24" s="10" t="inlineStr">
+      <c r="J25" s="10" t="inlineStr">
         <is>
           <t>STOP</t>
         </is>
       </c>
-      <c r="I24" s="9" t="n"/>
-      <c r="J24" s="9" t="n"/>
-      <c r="K24" s="9" t="n"/>
-      <c r="L24" s="9" t="n"/>
-      <c r="M24" s="9" t="n"/>
-      <c r="N24" s="9" t="n"/>
-      <c r="O24" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P24" s="13" t="inlineStr">
-        <is>
-          <t>PH proposal</t>
-        </is>
-      </c>
-      <c r="Q24" s="4" t="inlineStr">
-        <is>
-          <t>Works in AUTO and MAN. In AUTO the burner stays off until START is pressed.</t>
-        </is>
-      </c>
-      <c r="R24" s="14" t="n"/>
-      <c r="S24" s="15" t="n"/>
-    </row>
-    <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>C07j</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>BR01 running continuously for 24 h</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>Run timer &gt;= 24 h</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="G25" s="10" t="inlineStr">
-        <is>
-          <t>STOP</t>
-        </is>
-      </c>
-      <c r="H25" s="10" t="inlineStr">
-        <is>
-          <t>STOP</t>
-        </is>
-      </c>
-      <c r="I25" s="9" t="n"/>
-      <c r="J25" s="9" t="n"/>
       <c r="K25" s="9" t="n"/>
       <c r="L25" s="9" t="n"/>
       <c r="M25" s="9" t="n"/>
       <c r="N25" s="9" t="n"/>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>Automatic (restarts on next demand)</t>
-        </is>
-      </c>
-      <c r="P25" s="13" t="inlineStr">
-        <is>
-          <t>PH proposal</t>
+          <t>Automatic when level returns</t>
+        </is>
+      </c>
+      <c r="P25" s="16" t="inlineStr">
+        <is>
+          <t>Client</t>
         </is>
       </c>
       <c r="Q25" s="4" t="inlineStr">
         <is>
-          <t>RS100 is approved for intermittent operation and must stop at least once every 24 h (RS100 manual §5.10).</t>
+          <t>Client sheet: burner may run only when level has reached LSL. Contact closes with liquid present, so a broken wire also blocks the burner.</t>
         </is>
       </c>
       <c r="R25" s="14" t="n"/>
       <c r="S25" s="15" t="n"/>
     </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>BURNER BR02 — tank TK02</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="36" customHeight="1">
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>C08b</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>TE-503 / TE-504</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>TK02 oil temperature at setpoint</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>IW100 / IW102</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>max(T) &gt;= SP (70 °C)</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="9" t="n"/>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+      <c r="J26" s="10" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+      <c r="K26" s="9" t="n"/>
+      <c r="L26" s="9" t="n"/>
+      <c r="M26" s="9" t="n"/>
+      <c r="N26" s="9" t="n"/>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>Automatic at max(T) &lt;= SP − HYST (65 °C)</t>
+        </is>
+      </c>
+      <c r="P26" s="16" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="Q26" s="4" t="inlineStr">
+        <is>
+          <t>Client cases 2/3/6. The higher of inlet/outlet is used and the 5 °C restart band are PH proposals: each restart costs ~50 s of purge.</t>
+        </is>
+      </c>
+      <c r="R26" s="14" t="n"/>
+      <c r="S26" s="15" t="n"/>
+    </row>
+    <row r="27" ht="28" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>C08a</t>
+          <t>C08c</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>LSL-TK02</t>
+          <t>TE-503 / TE-504</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>TK02 level below low level switch (not ready)</t>
+          <t>TK02 oil temperature low — fast heat-up</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>I1.3</t>
+          <t>IW100 / IW102</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>LSL not reached (contact open)</t>
+          <t>max(T) &lt; SP − STG (60 °C)</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Permissive</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="G27" s="9" t="n"/>
       <c r="H27" s="9" t="n"/>
-      <c r="I27" s="10" t="inlineStr">
-        <is>
-          <t>STOP</t>
-        </is>
-      </c>
-      <c r="J27" s="10" t="inlineStr">
-        <is>
-          <t>STOP</t>
+      <c r="I27" s="9" t="n"/>
+      <c r="J27" s="17" t="inlineStr">
+        <is>
+          <t>RUN</t>
         </is>
       </c>
       <c r="K27" s="9" t="n"/>
@@ -2112,26 +2124,26 @@
       <c r="N27" s="9" t="n"/>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>Auto (AUTO mode)</t>
-        </is>
-      </c>
-      <c r="P27" s="16" t="inlineStr">
-        <is>
-          <t>Client</t>
+          <t>Automatic at max(T) &gt;= 60 °C</t>
+        </is>
+      </c>
+      <c r="P27" s="13" t="inlineStr">
+        <is>
+          <t>PH proposal</t>
         </is>
       </c>
       <c r="Q27" s="4" t="inlineStr">
         <is>
-          <t>Client sheet: burner may start only when level has reached LSL. Contact closes with liquid present, so a broken wire also blocks the burner.</t>
+          <t>2nd stage / high fire. Between 60 and 70 °C the burner runs on 1st stage.</t>
         </is>
       </c>
       <c r="R27" s="14" t="n"/>
       <c r="S27" s="15" t="n"/>
     </row>
-    <row r="28" ht="36" customHeight="1">
+    <row r="28" ht="28" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>C08b</t>
+          <t>C08d</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -2141,7 +2153,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>TK02 oil temperature at setpoint</t>
+          <t>Thermocouple fault — either of the two</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
@@ -2151,12 +2163,12 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>T &gt;= SP (70 °C)</t>
+          <t>Wire break or value out of range</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Trip</t>
         </is>
       </c>
       <c r="G28" s="9" t="n"/>
@@ -2174,71 +2186,83 @@
       <c r="K28" s="9" t="n"/>
       <c r="L28" s="9" t="n"/>
       <c r="M28" s="9" t="n"/>
-      <c r="N28" s="9" t="n"/>
+      <c r="N28" s="12" t="inlineStr">
+        <is>
+          <t>ALARM</t>
+        </is>
+      </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>Auto when T &lt;= SP − HYST (AUTO mode)</t>
-        </is>
-      </c>
-      <c r="P28" s="16" t="inlineStr">
-        <is>
-          <t>Client</t>
+          <t>S2 after fault cleared</t>
+        </is>
+      </c>
+      <c r="P28" s="13" t="inlineStr">
+        <is>
+          <t>PH proposal</t>
         </is>
       </c>
       <c r="Q28" s="4" t="inlineStr">
         <is>
-          <t>Client cases 2/3/6. Higher of inlet/outlet is used (PH proposal). Restart after hysteresis avoids short-cycling: each start costs ~50 s of purge.</t>
+          <t>Either sensor failing stops the burner: without both readings the higher value cannot be trusted.</t>
         </is>
       </c>
       <c r="R28" s="14" t="n"/>
       <c r="S28" s="15" t="n"/>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="36" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>C08c</t>
+          <t>C08e</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>TE-503 / TE-504</t>
+          <t>Rflt2</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>TK02 oil temperature below 2nd-stage threshold</t>
+          <t>BR02 lockout (flame / ignition / air pressure failure)</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>IW100 / IW102</t>
+          <t>I1.5</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>T &lt; SP − STG (60 °C)</t>
+          <t>Lockout signal present</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Trip</t>
         </is>
       </c>
       <c r="G29" s="9" t="n"/>
       <c r="H29" s="9" t="n"/>
-      <c r="I29" s="9" t="n"/>
-      <c r="J29" s="17" t="inlineStr">
-        <is>
-          <t>RUN</t>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+      <c r="J29" s="10" t="inlineStr">
+        <is>
+          <t>STOP</t>
         </is>
       </c>
       <c r="K29" s="9" t="n"/>
       <c r="L29" s="9" t="n"/>
       <c r="M29" s="9" t="n"/>
-      <c r="N29" s="9" t="n"/>
+      <c r="N29" s="12" t="inlineStr">
+        <is>
+          <t>ALARM</t>
+        </is>
+      </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>Auto when T &gt;= SP − STG</t>
+          <t>At burner control box, then S2</t>
         </is>
       </c>
       <c r="P29" s="13" t="inlineStr">
@@ -2248,7 +2272,7 @@
       </c>
       <c r="Q29" s="4" t="inlineStr">
         <is>
-          <t>Requests 2nd stage / high fire for fast heat-up. Between 60 and 70 °C: 1st stage only.</t>
+          <t>The burner's own control box has already closed the gas valves. PLC removes the heat request so the burner does not restart by itself after a local reset.</t>
         </is>
       </c>
       <c r="R29" s="14" t="n"/>
@@ -2257,27 +2281,27 @@
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>C08d</t>
+          <t>C08f</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>TE-503 / TE-504</t>
+          <t>RR2</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Thermocouple fault (wire break / out of range)</t>
+          <t>BR02 failed to start</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>IW100 / IW102</t>
+          <t>I1.4</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>SM 1231 diagnostic or value out of range</t>
+          <t>Heat request ON, no RUN within T_START (120 s)</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
@@ -2307,7 +2331,7 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>Manual (S2) after fault cleared</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="P30" s="13" t="inlineStr">
@@ -2317,7 +2341,7 @@
       </c>
       <c r="Q30" s="4" t="inlineStr">
         <is>
-          <t>Without a valid temperature the burner cannot be controlled.</t>
+          <t>RUN = gas valves energised (firing). Normal start ~55 s (RS100 §6.8.1) / ~65 s (DLX 53).</t>
         </is>
       </c>
       <c r="R30" s="14" t="n"/>
@@ -2326,32 +2350,32 @@
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>C08e</t>
+          <t>C08g</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Rflt2</t>
+          <t>RR2</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>BR02 burner lockout (flame failure, ignition failure, air pressure)</t>
+          <t>BR02 stopped by itself while running</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>I1.5</t>
+          <t>I1.4</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Lockout relay energised</t>
+          <t>RUN lost, no lockout, heat request still ON</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Alarm</t>
+          <t>Trip</t>
         </is>
       </c>
       <c r="G31" s="9" t="n"/>
@@ -2376,7 +2400,7 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>At burner control box, then S2</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="P31" s="13" t="inlineStr">
@@ -2386,411 +2410,37 @@
       </c>
       <c r="Q31" s="4" t="inlineStr">
         <is>
-          <t>Burner's own control box has already shut the gas valves. PLC removes the heat request so the burner does not restart by itself after a local reset.</t>
+          <t>E.g. safety thermostat TS, gas pressure switch, burner supply lost. Without this row the PLC would keep requesting heat from a burner that is no longer firing.</t>
         </is>
       </c>
       <c r="R31" s="14" t="n"/>
       <c r="S31" s="15" t="n"/>
     </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>C08f</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>RR2</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>BR02 failed to start</t>
-        </is>
-      </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>I1.4</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>Heat request ON and no RUN feedback within T_START (120 s)</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="inlineStr">
-        <is>
-          <t>Trip</t>
-        </is>
-      </c>
-      <c r="G32" s="9" t="n"/>
-      <c r="H32" s="9" t="n"/>
-      <c r="I32" s="10" t="inlineStr">
-        <is>
-          <t>STOP</t>
-        </is>
-      </c>
-      <c r="J32" s="10" t="inlineStr">
-        <is>
-          <t>STOP</t>
-        </is>
-      </c>
-      <c r="K32" s="9" t="n"/>
-      <c r="L32" s="9" t="n"/>
-      <c r="M32" s="9" t="n"/>
-      <c r="N32" s="12" t="inlineStr">
-        <is>
-          <t>ALARM</t>
-        </is>
-      </c>
-      <c r="O32" s="4" t="inlineStr">
-        <is>
-          <t>Manual (S2)</t>
-        </is>
-      </c>
-      <c r="P32" s="13" t="inlineStr">
-        <is>
-          <t>PH proposal</t>
-        </is>
-      </c>
-      <c r="Q32" s="4" t="inlineStr">
-        <is>
-          <t>Normal start cycle is ~55 s (RS100 manual §6.8.1) / ~65 s (DLX 53 manual).</t>
-        </is>
-      </c>
-      <c r="R32" s="14" t="n"/>
-      <c r="S32" s="15" t="n"/>
-    </row>
-    <row r="33" ht="48" customHeight="1">
-      <c r="A33" s="9" t="inlineStr">
-        <is>
-          <t>C08g</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>S5</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>BR02 selector in MANUAL</t>
-        </is>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>I12.2</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>Selector open = MAN</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
-        <is>
-          <t>Mode</t>
-        </is>
-      </c>
-      <c r="G33" s="9" t="n"/>
-      <c r="H33" s="9" t="n"/>
-      <c r="I33" s="9" t="n"/>
-      <c r="J33" s="9" t="n"/>
-      <c r="K33" s="9" t="n"/>
-      <c r="L33" s="9" t="n"/>
-      <c r="M33" s="9" t="n"/>
-      <c r="N33" s="9" t="n"/>
-      <c r="O33" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P33" s="16" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="Q33" s="4" t="inlineStr">
-        <is>
-          <t>Client e-mail: Auto/Manual selection. MAN: operator starts with START and stops with STOP. All trips and the temperature setpoint (C08b) still apply; no automatic restart.</t>
-        </is>
-      </c>
-      <c r="R33" s="14" t="n"/>
-      <c r="S33" s="15" t="n"/>
-    </row>
-    <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>C08h</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>S6</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>BR02 START push button (MAN mode)</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>I12.3</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>Pressed</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
-        <is>
-          <t>Command</t>
-        </is>
-      </c>
-      <c r="G34" s="9" t="n"/>
-      <c r="H34" s="9" t="n"/>
-      <c r="I34" s="17" t="inlineStr">
-        <is>
-          <t>RUN</t>
-        </is>
-      </c>
-      <c r="J34" s="9" t="n"/>
-      <c r="K34" s="9" t="n"/>
-      <c r="L34" s="9" t="n"/>
-      <c r="M34" s="9" t="n"/>
-      <c r="N34" s="9" t="n"/>
-      <c r="O34" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P34" s="13" t="inlineStr">
-        <is>
-          <t>PH proposal</t>
-        </is>
-      </c>
-      <c r="Q34" s="4" t="inlineStr">
-        <is>
-          <t>MAN: starts the burner. AUTO: re-enables automatic control after STOP. Ignored while any trip or permissive is active.</t>
-        </is>
-      </c>
-      <c r="R34" s="14" t="n"/>
-      <c r="S34" s="15" t="n"/>
-    </row>
-    <row r="35" ht="28" customHeight="1">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>C08i</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>S7</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>BR02 STOP push button</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>I12.4</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>Pressed</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>Command</t>
-        </is>
-      </c>
-      <c r="G35" s="9" t="n"/>
-      <c r="H35" s="9" t="n"/>
-      <c r="I35" s="10" t="inlineStr">
-        <is>
-          <t>STOP</t>
-        </is>
-      </c>
-      <c r="J35" s="10" t="inlineStr">
-        <is>
-          <t>STOP</t>
-        </is>
-      </c>
-      <c r="K35" s="9" t="n"/>
-      <c r="L35" s="9" t="n"/>
-      <c r="M35" s="9" t="n"/>
-      <c r="N35" s="9" t="n"/>
-      <c r="O35" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P35" s="13" t="inlineStr">
-        <is>
-          <t>PH proposal</t>
-        </is>
-      </c>
-      <c r="Q35" s="4" t="inlineStr">
-        <is>
-          <t>Works in AUTO and MAN. In AUTO the burner stays off until START is pressed.</t>
-        </is>
-      </c>
-      <c r="R35" s="14" t="n"/>
-      <c r="S35" s="15" t="n"/>
-    </row>
-    <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>C08j</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Rfuel2</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>BR02 in diesel mode</t>
-        </is>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>I12.0</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>Relay energised</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>Indication</t>
-        </is>
-      </c>
-      <c r="G36" s="9" t="n"/>
-      <c r="H36" s="9" t="n"/>
-      <c r="I36" s="9" t="n"/>
-      <c r="J36" s="9" t="n"/>
-      <c r="K36" s="9" t="n"/>
-      <c r="L36" s="9" t="n"/>
-      <c r="M36" s="9" t="n"/>
-      <c r="N36" s="9" t="n"/>
-      <c r="O36" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P36" s="16" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="Q36" s="4" t="inlineStr">
-        <is>
-          <t>Read only: fuel is selected on the burner itself. Shown on HMI.</t>
-        </is>
-      </c>
-      <c r="R36" s="14" t="n"/>
-      <c r="S36" s="15" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="9" t="inlineStr">
-        <is>
-          <t>C09</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>FAULT RESET push button</t>
-        </is>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>I1.1</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>Pressed</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="inlineStr">
-        <is>
-          <t>Command</t>
-        </is>
-      </c>
-      <c r="G38" s="9" t="n"/>
-      <c r="H38" s="9" t="n"/>
-      <c r="I38" s="9" t="n"/>
-      <c r="J38" s="9" t="n"/>
-      <c r="K38" s="9" t="n"/>
-      <c r="L38" s="9" t="n"/>
-      <c r="M38" s="9" t="n"/>
-      <c r="N38" s="9" t="n"/>
-      <c r="O38" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P38" s="13" t="inlineStr">
-        <is>
-          <t>PH proposal</t>
-        </is>
-      </c>
-      <c r="Q38" s="4" t="inlineStr">
-        <is>
-          <t>Resets latched trips only when their cause has cleared.</t>
-        </is>
-      </c>
-      <c r="R38" s="14" t="n"/>
-      <c r="S38" s="15" t="n"/>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
-  <autoFilter ref="A6:S38"/>
-  <mergeCells count="19">
+  <autoFilter ref="A6:S31"/>
+  <mergeCells count="18">
     <mergeCell ref="D4:D6"/>
+    <mergeCell ref="G4:N4"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="O4:O6"/>
+    <mergeCell ref="P4:P6"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="Q4:Q6"/>
+    <mergeCell ref="R4:R6"/>
+    <mergeCell ref="S4:S6"/>
+    <mergeCell ref="A7:S7"/>
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="E4:E6"/>
     <mergeCell ref="A10:S10"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="S4:S6"/>
+    <mergeCell ref="A24:S24"/>
+    <mergeCell ref="A2:S2"/>
+    <mergeCell ref="C4:C6"/>
     <mergeCell ref="A15:S15"/>
     <mergeCell ref="F4:F6"/>
-    <mergeCell ref="P4:P6"/>
-    <mergeCell ref="R4:R6"/>
-    <mergeCell ref="A1:S1"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="A7:S7"/>
-    <mergeCell ref="G4:N4"/>
-    <mergeCell ref="O4:O6"/>
-    <mergeCell ref="A37:S37"/>
-    <mergeCell ref="Q4:Q6"/>
-    <mergeCell ref="A26:S26"/>
-    <mergeCell ref="A2:S2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="R8 R9 R11 R12 R13 R14 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose Approved, Approved with comment or Rejected" prompt="Approved / Approved with comment / Rejected" type="list">
+    <dataValidation sqref="R8 R9 R11 R12 R13 R14 R16 R17 R18 R19 R20 R21 R22 R23 R25 R26 R27 R28 R29 R30 R31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose Approved, Approved with comment or Rejected" prompt="Approved / Approved with comment / Rejected" type="list">
       <formula1>"Approved,Approved with comment,Rejected"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(ce): 24 h stop is a permissive; type legend on the cover
</commit_message>
<xml_diff>
--- a/deliverables/PH-LCP-01-CE_RevA.xlsx
+++ b/deliverables/PH-LCP-01-CE_RevA.xlsx
@@ -664,7 +664,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="99" customHeight="1">
+    <row r="10" ht="138" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>How to read the matrix</t>
@@ -675,6 +675,7 @@
           <t>One row per cause. Cells under each effect say what happens to that output while the cause is active. Empty = no action.
 STOP = output de-energised / burner request removed.  RUN = energised.
 OPEN / CLOSE = resulting valve position.  ALARM = HMI alarm (the burner fault lamps H3 / H4 are wired to the burner lockout, not to the PLC).
+Type: Trip = stops and stays stopped until RESET (S2).  Permissive = stops, restarts by itself when the condition clears.  Control = normal temperature regulation.  Alarm = HMI message only.  Inherent = happens by wiring, no program.
 Column 'Source' shows where each line comes from: Client = client document; PH proposal = proposed by PH, to be approved by the client.</t>
         </is>
       </c>
@@ -1905,7 +1906,7 @@
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Permissive</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">

</xml_diff>

<commit_message>
fix(ce): cover fits one page again
</commit_message>
<xml_diff>
--- a/deliverables/PH-LCP-01-CE_RevA.xlsx
+++ b/deliverables/PH-LCP-01-CE_RevA.xlsx
@@ -591,7 +591,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="34" customHeight="1">
+    <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Purpose</t>
@@ -603,7 +603,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="47" customHeight="1">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Scope</t>
@@ -615,7 +615,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="47" customHeight="1">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Not in scope (Rev. A)</t>
@@ -628,7 +628,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="47" customHeight="1">
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Burner flame safety</t>
@@ -640,7 +640,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="34" customHeight="1">
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Hardwired safety</t>
@@ -652,7 +652,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="34" customHeight="1">
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Fail-safe outputs</t>
@@ -664,7 +664,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="138" customHeight="1">
+    <row r="10" ht="114" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>How to read the matrix</t>
@@ -680,7 +680,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1">
+    <row r="11" ht="42" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Requested from client</t>

</xml_diff>

<commit_message>
docs: apply verified Codex review — rules R-01..R-12, F17–F30
راجعت كل ملاحظة من مراجعة Codex على الملفات قبل ما أقبلها، وكلها
طلعت صح:
- الثيرموكابل: كل قناة تتراجع قبل MAX، و−32768 كمان (F17).
- STOP والشروط بيقفلوا من STARTING كمان، وفيه أولوية (F19).
- E-STOP بيروح FAULT ومحتاج RESET، وSTART وRESET على الحافة (F22).
- وقفة الـ 24 ساعة 60 ثانية مؤكدة (F21).
- قطبية S3 NC اتكتبت (F20)، والمخارج OFF عند STOP (F23).
- تصنيف PH decision بدل Client للي إحنا قررناه (F26).
- التشغيل.md §8: 12 قاعدة للمواقف اللي مكانتش متعرّفة.
فاضل للموقع: F18 (حماية حرارة TK02)، وF20 (S7)، وF25 (BR02)، وF30.
وللأدوات: F28 وF29.
</commit_message>
<xml_diff>
--- a/deliverables/PH-LCP-01-CE_RevA.xlsx
+++ b/deliverables/PH-LCP-01-CE_RevA.xlsx
@@ -61,7 +61,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -110,6 +110,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
@@ -145,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -197,7 +202,10 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -675,8 +683,8 @@
           <t>One row per cause. Cells under each effect say what happens to that output while the cause is active. Empty = no action.
 STOP = output de-energised / burner request removed.  RUN = energised.
 OPEN / CLOSE = resulting valve position.  ALARM = HMI alarm (the burner fault lamps H3 / H4 are wired to the burner lockout, not to the PLC).
-Type: Trip = stops and stays stopped until RESET (S2).  Permissive = stops, restarts by itself when the condition clears.  Control = normal temperature regulation.  Alarm = HMI message only.  Inherent = happens by wiring, no program.
-Column 'Source' shows where each line comes from: Client = client document; PH proposal = proposed by PH, to be approved by the client.</t>
+Type: Trip = stops and stays stopped until RESET (S2).  Permissive = stops, restarts by itself when the condition clears (AUTO mode, burner enabled).  Control = normal temperature regulation.  Alarm = HMI message only.  Inherent = happens by wiring, no program.
+Column 'Source': Client = client document; PH decision = decided by PH (Eng. Ahmed Zain); PH proposal = proposed by PH, still open.</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1148,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="48" customHeight="1">
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
           <t>C03</t>
@@ -1202,12 +1210,12 @@
       </c>
       <c r="P11" s="16" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>PH decision</t>
         </is>
       </c>
       <c r="Q11" s="4" t="inlineStr">
         <is>
-          <t>Client e-mail: scrubber alarms/trips. Burners are NOT tripped (decision PH / Eng. Ahmed Zain); if gas pressure to the burner drops, the burner's own gas pressure switch stops it (C07g / C08g).</t>
+          <t>Client e-mail asks for scrubber alarms/trips; the valve action and burner policy were decided by PH. Burners are NOT tripped (decision PH / Eng. Ahmed Zain); if gas pressure to the burner drops, the burner's own gas pressure switch stops it (C07g / C08g).</t>
         </is>
       </c>
       <c r="R11" s="14" t="n"/>
@@ -1261,7 +1269,7 @@
           <t>Automatic when cleared</t>
         </is>
       </c>
-      <c r="P12" s="16" t="inlineStr">
+      <c r="P12" s="17" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -1336,7 +1344,7 @@
       </c>
       <c r="P13" s="16" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>PH decision</t>
         </is>
       </c>
       <c r="Q13" s="4" t="inlineStr">
@@ -1393,12 +1401,12 @@
       </c>
       <c r="P14" s="16" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>PH decision</t>
         </is>
       </c>
       <c r="Q14" s="4" t="inlineStr">
         <is>
-          <t>Not installed — excluded from Rev. A. Input reserved for future use.</t>
+          <t>Provisional: understood as not installed (open question Q1). Input reserved.</t>
         </is>
       </c>
       <c r="R14" s="14" t="n"/>
@@ -1463,7 +1471,7 @@
           <t>Automatic when level returns</t>
         </is>
       </c>
-      <c r="P16" s="16" t="inlineStr">
+      <c r="P16" s="17" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -1528,7 +1536,7 @@
           <t>Automatic at max(T) &lt;= SP − HYST (65 °C)</t>
         </is>
       </c>
-      <c r="P17" s="16" t="inlineStr">
+      <c r="P17" s="17" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -1573,7 +1581,7 @@
         </is>
       </c>
       <c r="G18" s="9" t="n"/>
-      <c r="H18" s="17" t="inlineStr">
+      <c r="H18" s="18" t="inlineStr">
         <is>
           <t>RUN</t>
         </is>
@@ -1602,7 +1610,7 @@
       <c r="R18" s="14" t="n"/>
       <c r="S18" s="15" t="n"/>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="48" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
         <is>
           <t>C07d</t>
@@ -1625,7 +1633,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Wire break or value out of range</t>
+          <t>Either channel: 32767 / −32768, outside −20…150 °C, or channel diagnostic</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
@@ -1665,7 +1673,7 @@
       </c>
       <c r="Q19" s="4" t="inlineStr">
         <is>
-          <t>Either sensor failing stops the burner: without both readings the higher value cannot be trusted.</t>
+          <t>Each channel is checked BEFORE taking the higher value, so one failed-low sensor cannot hide behind the other. Heat is inhibited until both channels are valid after power-up.</t>
         </is>
       </c>
       <c r="R19" s="14" t="n"/>
@@ -2002,7 +2010,7 @@
           <t>Automatic when level returns</t>
         </is>
       </c>
-      <c r="P25" s="16" t="inlineStr">
+      <c r="P25" s="17" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -2067,7 +2075,7 @@
           <t>Automatic at max(T) &lt;= SP − HYST (65 °C)</t>
         </is>
       </c>
-      <c r="P26" s="16" t="inlineStr">
+      <c r="P26" s="17" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
@@ -2114,7 +2122,7 @@
       <c r="G27" s="9" t="n"/>
       <c r="H27" s="9" t="n"/>
       <c r="I27" s="9" t="n"/>
-      <c r="J27" s="17" t="inlineStr">
+      <c r="J27" s="18" t="inlineStr">
         <is>
           <t>RUN</t>
         </is>
@@ -2141,7 +2149,7 @@
       <c r="R27" s="14" t="n"/>
       <c r="S27" s="15" t="n"/>
     </row>
-    <row r="28" ht="28" customHeight="1">
+    <row r="28" ht="48" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
           <t>C08d</t>
@@ -2164,7 +2172,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Wire break or value out of range</t>
+          <t>Either channel: 32767 / −32768, outside −20…150 °C, or channel diagnostic</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
@@ -2204,7 +2212,7 @@
       </c>
       <c r="Q28" s="4" t="inlineStr">
         <is>
-          <t>Either sensor failing stops the burner: without both readings the higher value cannot be trusted.</t>
+          <t>Each channel is checked BEFORE taking the higher value, so one failed-low sensor cannot hide behind the other. Heat is inhibited until both channels are valid after power-up.</t>
         </is>
       </c>
       <c r="R28" s="14" t="n"/>
@@ -2524,7 +2532,7 @@
           <t>Tank temperature setpoint — burner stops at T &gt;= SP</t>
         </is>
       </c>
-      <c r="C5" s="18" t="n">
+      <c r="C5" s="19" t="n">
         <v>70</v>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -2554,7 +2562,7 @@
           <t>Restart hysteresis — burner restarts at T &lt;= SP − HYST</t>
         </is>
       </c>
-      <c r="C6" s="18" t="n">
+      <c r="C6" s="19" t="n">
         <v>5</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -2584,7 +2592,7 @@
           <t>2nd stage / high fire while T &lt; SP − STG</t>
         </is>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="C7" s="19" t="n">
         <v>10</v>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -2614,7 +2622,7 @@
           <t>Max. time from heat request to RUN feedback</t>
         </is>
       </c>
-      <c r="C8" s="18" t="n">
+      <c r="C8" s="19" t="n">
         <v>120</v>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -2644,7 +2652,7 @@
           <t>Forced stop of BR01 after continuous run</t>
         </is>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="9" t="n">
         <v>24</v>
       </c>
       <c r="D9" s="9" t="inlineStr">

</xml_diff>

<commit_message>
fix(ce): name buttons and relays next to their codes
</commit_message>
<xml_diff>
--- a/deliverables/PH-LCP-01-CE_RevA.xlsx
+++ b/deliverables/PH-LCP-01-CE_RevA.xlsx
@@ -975,7 +975,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>S0</t>
+          <t>S0 (E-STOP)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>Release S0, then S2; burners need START</t>
+          <t>Release S0 (E-STOP), then S2 (RESET); burners need START (S1 / S6)</t>
         </is>
       </c>
       <c r="P8" s="13" t="inlineStr">
@@ -1125,7 +1125,7 @@
       <c r="N9" s="9" t="n"/>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>S2 for scrubber; burners need START</t>
+          <t>S2 (RESET) for scrubber; burners need START (S1 / S6)</t>
         </is>
       </c>
       <c r="P9" s="13" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>S2 after cleared</t>
+          <t>S2 (RESET) after cleared</t>
         </is>
       </c>
       <c r="P11" s="16" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>S2 after cleared</t>
+          <t>S2 (RESET) after cleared</t>
         </is>
       </c>
       <c r="P13" s="16" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>S2 after fault cleared</t>
+          <t>S2 (RESET) after fault cleared</t>
         </is>
       </c>
       <c r="P19" s="13" t="inlineStr">
@@ -1687,7 +1687,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Rflt</t>
+          <t>Rflt (BR01 fault relay)</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>At burner control box, then S2</t>
+          <t>At burner control box, then S2 (RESET)</t>
         </is>
       </c>
       <c r="P20" s="13" t="inlineStr">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RR (BR01 run relay)</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S2 (RESET)</t>
         </is>
       </c>
       <c r="P21" s="13" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RR (BR01 run relay)</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S2 (RESET)</t>
         </is>
       </c>
       <c r="P22" s="13" t="inlineStr">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>S2 after fault cleared</t>
+          <t>S2 (RESET) after fault cleared</t>
         </is>
       </c>
       <c r="P28" s="13" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Rflt2</t>
+          <t>Rflt2 (BR02 fault relay)</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>At burner control box, then S2</t>
+          <t>At burner control box, then S2 (RESET)</t>
         </is>
       </c>
       <c r="P29" s="13" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>RR2</t>
+          <t>RR2 (BR02 run relay)</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S2 (RESET)</t>
         </is>
       </c>
       <c r="P30" s="13" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>RR2</t>
+          <t>RR2 (BR02 run relay)</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S2 (RESET)</t>
         </is>
       </c>
       <c r="P31" s="13" t="inlineStr">

</xml_diff>

<commit_message>
feat(tools): generate the PLC tag table from the IO List and import it
الـ IO List بقى فيه عمود PLC Tag (31 اسم حسب 0005). build_tags.py بيطلّع
build/tags/IO.xml، وApply-Tags.ps1 بيستورده ويعمل compile ويحفظ بس لو نضيف.
Codex (gpt-6-luna) كتبه، واتراجع هنا. الفحوصات عدّت، والاستيراد على المشروع
بـ DryRun طلع errors 0 (مااتحفظش). الأسماء اللي فيها اختيار مستنية تأكيد
المستخدم: evidence/2026-10-28-tag-table-dryrun.md.
</commit_message>
<xml_diff>
--- a/deliverables/PH-LCP-01-CE_RevA.xlsx
+++ b/deliverables/PH-LCP-01-CE_RevA.xlsx
@@ -2695,7 +2695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2704,6 +2704,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -2751,6 +2752,11 @@
           <t>Sheet</t>
         </is>
       </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>PLC Tag</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -2783,6 +2789,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>PSH_101</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -2815,6 +2826,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>LSH_102</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -2847,6 +2863,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>LSHH_103</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -2879,6 +2900,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>BR01_Run</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -2911,6 +2937,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>S1_BR01_Start</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -2943,6 +2974,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>BR01_Fault</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -2975,6 +3011,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>S3_BR01_Stop</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -3007,6 +3048,7 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -3039,6 +3081,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>S0_EStopStatus</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -3071,6 +3118,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>S2_FaultReset</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -3103,6 +3155,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>LSL_TK01</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -3135,6 +3192,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>LSL_TK02</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -3167,6 +3229,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>BR02_Run</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -3199,6 +3266,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>BR02_Fault</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -3231,6 +3303,11 @@
           <t>11</t>
         </is>
       </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Rfuel2_BR02_DieselMode</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -3263,6 +3340,11 @@
           <t>11</t>
         </is>
       </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>S4_BR01_Auto</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
@@ -3295,6 +3377,11 @@
           <t>11</t>
         </is>
       </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>S5_BR02_Auto</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
@@ -3327,6 +3414,11 @@
           <t>11</t>
         </is>
       </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>S6_BR02_Start</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
@@ -3359,6 +3451,11 @@
           <t>11</t>
         </is>
       </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>S7_BR02_Stop</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
@@ -3391,6 +3488,7 @@
           <t>11</t>
         </is>
       </c>
+      <c r="G24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
@@ -3423,6 +3521,7 @@
           <t>11</t>
         </is>
       </c>
+      <c r="G25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
@@ -3455,6 +3554,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>BR01_TL_Cmd</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
@@ -3487,6 +3591,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>BR01_TR_Cmd</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
@@ -3519,6 +3628,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>XV_401_Cmd</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
@@ -3551,6 +3665,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>XV_402_Cmd</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
@@ -3583,6 +3702,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>XV_403_Cmd</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
@@ -3615,6 +3739,11 @@
           <t>12 / 8</t>
         </is>
       </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>BR02_L_Cmd</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
@@ -3647,6 +3776,11 @@
           <t>12 / 8</t>
         </is>
       </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>BR02_T2_Cmd</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
@@ -3679,6 +3813,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>BR02_Stage1Lamp_Cmd</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
@@ -3711,6 +3850,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>BR02_Stage2Lamp_Cmd</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
@@ -3743,6 +3887,7 @@
           <t>12</t>
         </is>
       </c>
+      <c r="G35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
@@ -3775,6 +3920,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>TE_501_Raw</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
@@ -3807,6 +3957,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>TE_502_Raw</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
@@ -3839,6 +3994,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>TE_503_Raw</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
@@ -3871,6 +4031,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>TE_504_Raw</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
@@ -3903,11 +4068,12 @@
           <t>13</t>
         </is>
       </c>
+      <c r="G40" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
feat(tia): 2 degC band on the 2nd stage (F41)
المستخدم اختار فرق درجتين: المرحلة التانية ON تحت SP-STG (60) و OFF عند 62،
عشان R2/R7 مايقلبوش عند 60. اتعدّل C07c/C08c في الـ C&E (لسه PH proposal)،
و التشغيل.md §2، و Burner FB، و اختبار T1. لسه مااتعملش import (TIA مفتوح).
</commit_message>
<xml_diff>
--- a/deliverables/PH-LCP-01-CE_RevA.xlsx
+++ b/deliverables/PH-LCP-01-CE_RevA.xlsx
@@ -1549,7 +1549,7 @@
       <c r="R17" s="14" t="n"/>
       <c r="S17" s="15" t="n"/>
     </row>
-    <row r="18" ht="28" customHeight="1">
+    <row r="18" ht="36" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
           <t>C07c</t>
@@ -1594,7 +1594,7 @@
       <c r="N18" s="9" t="n"/>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>Automatic at max(T) &gt;= 60 °C</t>
+          <t>Automatic at max(T) &gt;= 62 °C (2 °C band)</t>
         </is>
       </c>
       <c r="P18" s="13" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="Q18" s="4" t="inlineStr">
         <is>
-          <t>2nd stage / high fire. Between 60 and 70 °C the burner runs on 1st stage.</t>
+          <t>2nd stage / high fire. Between 60 and 70 °C the burner runs on 1st stage. Back to 1st stage at 62 °C: the 2 °C band stops relay R2 / R7 chattering at 60 °C.</t>
         </is>
       </c>
       <c r="R18" s="14" t="n"/>
@@ -2088,7 +2088,7 @@
       <c r="R26" s="14" t="n"/>
       <c r="S26" s="15" t="n"/>
     </row>
-    <row r="27" ht="28" customHeight="1">
+    <row r="27" ht="36" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
           <t>C08c</t>
@@ -2133,7 +2133,7 @@
       <c r="N27" s="9" t="n"/>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>Automatic at max(T) &gt;= 60 °C</t>
+          <t>Automatic at max(T) &gt;= 62 °C (2 °C band)</t>
         </is>
       </c>
       <c r="P27" s="13" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="Q27" s="4" t="inlineStr">
         <is>
-          <t>2nd stage / high fire. Between 60 and 70 °C the burner runs on 1st stage.</t>
+          <t>2nd stage / high fire. Between 60 and 70 °C the burner runs on 1st stage. Back to 1st stage at 62 °C: the 2 °C band stops relay R2 / R7 chattering at 60 °C.</t>
         </is>
       </c>
       <c r="R27" s="14" t="n"/>

</xml_diff>